<commit_message>
Blinkit statewise: add RO Accepted Qty from Bulk RO acceptance caps
Reads Blinkit's SELLER_BULK_SHIPMENT_INPUT.xlsx (Bulk RO sheet) to compute
per-(item, state) headroom = max(0, Max Inventory - Sellable - Incoming),
excluding LOCKED warehouse lines. Adds two columns to the per-state view:
  - ro_headroom        — what Blinkit will physically accept in that state
  - ro_accepted_qty    — min(state_deficiency, ro_headroom), gated to only
                         populate where state_deficiency > 0

Also refreshes the Blinkit inventory + monthly sales (Mar/Apr/May 2026).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Blinkit/Inventory/InventoryData.xlsx
+++ b/data/input/Blinkit/Inventory/InventoryData.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_39B8DDE40B346ACAF331DDD578760E63E6F0ED56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Stock On Hand" sheetId="2" r:id="rId4"/>
+    <sheet name="Stock On Hand" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1638" uniqueCount="172">
   <si>
     <t>Product details</t>
   </si>
@@ -535,7 +536,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -544,14 +545,14 @@
       <family val="2"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
       <name val="Proxima Nova"/>
       <family val="2"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Proxima Nova"/>
@@ -633,30 +634,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -664,12 +668,20 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -924,147 +936,148 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:W271"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="15"/>
-    <col customWidth="true" max="2" min="2" width="75"/>
-    <col customWidth="true" max="3" min="3" width="16"/>
-    <col customWidth="true" max="4" min="4" width="15"/>
-    <col customWidth="true" max="5" min="5" width="8"/>
-    <col customWidth="true" max="6" min="6" width="23"/>
-    <col customWidth="true" max="7" min="7" width="28"/>
-    <col customWidth="true" max="8" min="8" width="25"/>
-    <col customWidth="true" max="9" min="9" width="30"/>
-    <col customWidth="true" max="10" min="10" width="20"/>
-    <col customWidth="true" max="11" min="11" width="16"/>
-    <col customWidth="true" max="12" min="12" width="11"/>
-    <col customWidth="true" max="13" min="13" width="12"/>
-    <col customWidth="true" max="14" min="14" width="11"/>
-    <col customWidth="true" max="15" min="15" width="18"/>
-    <col customWidth="true" max="16" min="16" width="9"/>
-    <col customWidth="true" max="17" min="17" width="6"/>
-    <col customWidth="true" max="18" min="18" width="9"/>
-    <col customWidth="true" max="20" min="19" width="13"/>
-    <col customWidth="true" max="22" min="21" width="14"/>
-    <col customWidth="true" max="23" min="23" width="9"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="75" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="9" customWidth="1"/>
+    <col min="17" max="17" width="6" customWidth="1"/>
+    <col min="18" max="18" width="9" customWidth="1"/>
+    <col min="19" max="20" width="13" customWidth="1"/>
+    <col min="21" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:23">
       <c r="A1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="2" ht="35" customHeight="true">
-      <c r="A2" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="1" t="s">
+    <row r="2" spans="1:23" ht="34.950000000000003" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="5" t="s">
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="6" t="s">
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="7" t="s">
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="7"/>
-      <c r="V2" s="7"/>
-      <c r="W2" s="2" t="s">
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:23" ht="15.6">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="U3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="W3" s="2"/>
-    </row>
-    <row r="4">
+      <c r="W3" s="9"/>
+    </row>
+    <row r="4" spans="1:23">
       <c r="A4">
         <v>10222298</v>
       </c>
@@ -1135,7 +1148,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:23">
       <c r="A5">
         <v>10222298</v>
       </c>
@@ -1206,7 +1219,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:23">
       <c r="A6">
         <v>10222298</v>
       </c>
@@ -1277,7 +1290,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:23">
       <c r="A7">
         <v>10222298</v>
       </c>
@@ -1348,7 +1361,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:23">
       <c r="A8">
         <v>10222298</v>
       </c>
@@ -1419,7 +1432,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:23">
       <c r="A9">
         <v>10222298</v>
       </c>
@@ -1490,7 +1503,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:23">
       <c r="A10">
         <v>10222298</v>
       </c>
@@ -1561,7 +1574,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:23">
       <c r="A11">
         <v>10222298</v>
       </c>
@@ -1632,7 +1645,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:23">
       <c r="A12">
         <v>10222298</v>
       </c>
@@ -1703,7 +1716,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:23">
       <c r="A13">
         <v>10222298</v>
       </c>
@@ -1774,7 +1787,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:23">
       <c r="A14">
         <v>10222298</v>
       </c>
@@ -1845,7 +1858,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:23">
       <c r="A15">
         <v>10222298</v>
       </c>
@@ -1916,7 +1929,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:23">
       <c r="A16">
         <v>10222298</v>
       </c>
@@ -1987,7 +2000,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:23">
       <c r="A17">
         <v>10222298</v>
       </c>
@@ -2058,7 +2071,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:23">
       <c r="A18">
         <v>10222298</v>
       </c>
@@ -2129,7 +2142,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:23">
       <c r="A19">
         <v>10222304</v>
       </c>
@@ -2200,7 +2213,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:23">
       <c r="A20">
         <v>10222304</v>
       </c>
@@ -2271,7 +2284,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:23">
       <c r="A21">
         <v>10222304</v>
       </c>
@@ -2342,7 +2355,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:23">
       <c r="A22">
         <v>10222304</v>
       </c>
@@ -2413,7 +2426,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:23">
       <c r="A23">
         <v>10222304</v>
       </c>
@@ -2484,7 +2497,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:23">
       <c r="A24">
         <v>10222304</v>
       </c>
@@ -2555,7 +2568,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:23">
       <c r="A25">
         <v>10222304</v>
       </c>
@@ -2626,7 +2639,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:23">
       <c r="A26">
         <v>10222304</v>
       </c>
@@ -2697,7 +2710,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:23">
       <c r="A27">
         <v>10222304</v>
       </c>
@@ -2768,7 +2781,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:23">
       <c r="A28">
         <v>10222304</v>
       </c>
@@ -2839,7 +2852,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:23">
       <c r="A29">
         <v>10222304</v>
       </c>
@@ -2910,7 +2923,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:23">
       <c r="A30">
         <v>10222304</v>
       </c>
@@ -2981,7 +2994,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:23">
       <c r="A31">
         <v>10222304</v>
       </c>
@@ -3052,7 +3065,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:23">
       <c r="A32">
         <v>10223639</v>
       </c>
@@ -3123,7 +3136,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:23">
       <c r="A33">
         <v>10223639</v>
       </c>
@@ -3194,7 +3207,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:23">
       <c r="A34">
         <v>10223639</v>
       </c>
@@ -3265,7 +3278,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:23">
       <c r="A35">
         <v>10223639</v>
       </c>
@@ -3336,7 +3349,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:23">
       <c r="A36">
         <v>10223639</v>
       </c>
@@ -3407,7 +3420,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:23">
       <c r="A37">
         <v>10223639</v>
       </c>
@@ -3478,7 +3491,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:23">
       <c r="A38">
         <v>10223639</v>
       </c>
@@ -3549,7 +3562,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:23">
       <c r="A39">
         <v>10223639</v>
       </c>
@@ -3620,7 +3633,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:23">
       <c r="A40">
         <v>10223639</v>
       </c>
@@ -3691,7 +3704,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:23">
       <c r="A41">
         <v>10223872</v>
       </c>
@@ -3762,7 +3775,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:23">
       <c r="A42">
         <v>10223872</v>
       </c>
@@ -3833,7 +3846,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:23">
       <c r="A43">
         <v>10224530</v>
       </c>
@@ -3904,7 +3917,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:23">
       <c r="A44">
         <v>10224530</v>
       </c>
@@ -3975,7 +3988,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:23">
       <c r="A45">
         <v>10224530</v>
       </c>
@@ -4046,7 +4059,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:23">
       <c r="A46">
         <v>10224530</v>
       </c>
@@ -4117,7 +4130,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:23">
       <c r="A47">
         <v>10224530</v>
       </c>
@@ -4188,7 +4201,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:23">
       <c r="A48">
         <v>10224530</v>
       </c>
@@ -4259,7 +4272,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:23">
       <c r="A49">
         <v>10224530</v>
       </c>
@@ -4330,7 +4343,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:23">
       <c r="A50">
         <v>10224530</v>
       </c>
@@ -4401,7 +4414,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:23">
       <c r="A51">
         <v>10224530</v>
       </c>
@@ -4472,7 +4485,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:23">
       <c r="A52">
         <v>10225087</v>
       </c>
@@ -4543,7 +4556,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:23">
       <c r="A53">
         <v>10225087</v>
       </c>
@@ -4614,7 +4627,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:23">
       <c r="A54">
         <v>10225087</v>
       </c>
@@ -4685,7 +4698,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:23">
       <c r="A55">
         <v>10225087</v>
       </c>
@@ -4756,7 +4769,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:23">
       <c r="A56">
         <v>10225457</v>
       </c>
@@ -4827,7 +4840,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:23">
       <c r="A57">
         <v>10225457</v>
       </c>
@@ -4898,7 +4911,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:23">
       <c r="A58">
         <v>10225457</v>
       </c>
@@ -4969,7 +4982,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:23">
       <c r="A59">
         <v>10225457</v>
       </c>
@@ -5040,7 +5053,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:23">
       <c r="A60">
         <v>10225457</v>
       </c>
@@ -5111,7 +5124,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:23">
       <c r="A61">
         <v>10225457</v>
       </c>
@@ -5182,7 +5195,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:23">
       <c r="A62">
         <v>10225457</v>
       </c>
@@ -5253,7 +5266,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:23">
       <c r="A63">
         <v>10225457</v>
       </c>
@@ -5324,7 +5337,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:23">
       <c r="A64">
         <v>10225457</v>
       </c>
@@ -5395,7 +5408,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:23">
       <c r="A65">
         <v>10225457</v>
       </c>
@@ -5466,7 +5479,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:23">
       <c r="A66">
         <v>10225457</v>
       </c>
@@ -5537,7 +5550,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:23">
       <c r="A67">
         <v>10226828</v>
       </c>
@@ -5608,7 +5621,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:23">
       <c r="A68">
         <v>10226828</v>
       </c>
@@ -5679,7 +5692,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:23">
       <c r="A69">
         <v>10226828</v>
       </c>
@@ -5750,7 +5763,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:23">
       <c r="A70">
         <v>10229301</v>
       </c>
@@ -5821,7 +5834,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:23">
       <c r="A71">
         <v>10229301</v>
       </c>
@@ -5892,7 +5905,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:23">
       <c r="A72">
         <v>10229301</v>
       </c>
@@ -5963,7 +5976,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:23">
       <c r="A73">
         <v>10229301</v>
       </c>
@@ -6034,7 +6047,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:23">
       <c r="A74">
         <v>10229301</v>
       </c>
@@ -6105,7 +6118,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:23">
       <c r="A75">
         <v>10229301</v>
       </c>
@@ -6176,7 +6189,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:23">
       <c r="A76">
         <v>10229301</v>
       </c>
@@ -6247,7 +6260,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:23">
       <c r="A77">
         <v>10229357</v>
       </c>
@@ -6318,7 +6331,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:23">
       <c r="A78">
         <v>10229357</v>
       </c>
@@ -6389,7 +6402,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:23">
       <c r="A79">
         <v>10229357</v>
       </c>
@@ -6460,7 +6473,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:23">
       <c r="A80">
         <v>10229357</v>
       </c>
@@ -6531,7 +6544,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:23">
       <c r="A81">
         <v>10229357</v>
       </c>
@@ -6602,7 +6615,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:23">
       <c r="A82">
         <v>10229357</v>
       </c>
@@ -6673,7 +6686,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:23">
       <c r="A83">
         <v>10229357</v>
       </c>
@@ -6744,7 +6757,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:23">
       <c r="A84">
         <v>10229357</v>
       </c>
@@ -6815,7 +6828,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:23">
       <c r="A85">
         <v>10229357</v>
       </c>
@@ -6886,7 +6899,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:23">
       <c r="A86">
         <v>10229357</v>
       </c>
@@ -6957,7 +6970,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:23">
       <c r="A87">
         <v>10229357</v>
       </c>
@@ -7028,7 +7041,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:23">
       <c r="A88">
         <v>10229879</v>
       </c>
@@ -7099,7 +7112,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:23">
       <c r="A89">
         <v>10229879</v>
       </c>
@@ -7170,7 +7183,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:23">
       <c r="A90">
         <v>10229879</v>
       </c>
@@ -7241,7 +7254,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:23">
       <c r="A91">
         <v>10229879</v>
       </c>
@@ -7312,7 +7325,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:23">
       <c r="A92">
         <v>10229879</v>
       </c>
@@ -7383,7 +7396,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:23">
       <c r="A93">
         <v>10229879</v>
       </c>
@@ -7454,7 +7467,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:23">
       <c r="A94">
         <v>10229879</v>
       </c>
@@ -7525,7 +7538,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:23">
       <c r="A95">
         <v>10229879</v>
       </c>
@@ -7596,7 +7609,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:23">
       <c r="A96">
         <v>10229879</v>
       </c>
@@ -7667,7 +7680,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:23">
       <c r="A97">
         <v>10232177</v>
       </c>
@@ -7738,7 +7751,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:23">
       <c r="A98">
         <v>10232177</v>
       </c>
@@ -7809,7 +7822,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:23">
       <c r="A99">
         <v>10232177</v>
       </c>
@@ -7880,7 +7893,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:23">
       <c r="A100">
         <v>10232177</v>
       </c>
@@ -7951,7 +7964,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:23">
       <c r="A101">
         <v>10232177</v>
       </c>
@@ -8022,7 +8035,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:23">
       <c r="A102">
         <v>10232177</v>
       </c>
@@ -8093,7 +8106,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:23">
       <c r="A103">
         <v>10232177</v>
       </c>
@@ -8164,7 +8177,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:23">
       <c r="A104">
         <v>10232177</v>
       </c>
@@ -8235,7 +8248,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:23">
       <c r="A105">
         <v>10234935</v>
       </c>
@@ -8306,7 +8319,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:23">
       <c r="A106">
         <v>10234935</v>
       </c>
@@ -8377,7 +8390,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:23">
       <c r="A107">
         <v>10234935</v>
       </c>
@@ -8448,7 +8461,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:23">
       <c r="A108">
         <v>10234935</v>
       </c>
@@ -8519,7 +8532,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:23">
       <c r="A109">
         <v>10234935</v>
       </c>
@@ -8590,7 +8603,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:23">
       <c r="A110">
         <v>10235460</v>
       </c>
@@ -8661,7 +8674,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:23">
       <c r="A111">
         <v>10235460</v>
       </c>
@@ -8732,7 +8745,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:23">
       <c r="A112">
         <v>10235460</v>
       </c>
@@ -8803,7 +8816,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:23">
       <c r="A113">
         <v>10235460</v>
       </c>
@@ -8874,7 +8887,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:23">
       <c r="A114">
         <v>10235460</v>
       </c>
@@ -8945,7 +8958,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:23">
       <c r="A115">
         <v>10235460</v>
       </c>
@@ -9016,7 +9029,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:23">
       <c r="A116">
         <v>10235473</v>
       </c>
@@ -9087,7 +9100,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:23">
       <c r="A117">
         <v>10235473</v>
       </c>
@@ -9158,7 +9171,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:23">
       <c r="A118">
         <v>10235473</v>
       </c>
@@ -9229,7 +9242,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:23">
       <c r="A119">
         <v>10235831</v>
       </c>
@@ -9300,7 +9313,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:23">
       <c r="A120">
         <v>10235831</v>
       </c>
@@ -9371,7 +9384,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:23">
       <c r="A121">
         <v>10235831</v>
       </c>
@@ -9442,7 +9455,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:23">
       <c r="A122">
         <v>10235831</v>
       </c>
@@ -9513,7 +9526,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:23">
       <c r="A123">
         <v>10235831</v>
       </c>
@@ -9584,7 +9597,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:23">
       <c r="A124">
         <v>10235849</v>
       </c>
@@ -9655,7 +9668,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:23">
       <c r="A125">
         <v>10235849</v>
       </c>
@@ -9726,7 +9739,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:23">
       <c r="A126">
         <v>10235849</v>
       </c>
@@ -9797,7 +9810,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:23">
       <c r="A127">
         <v>10235849</v>
       </c>
@@ -9868,7 +9881,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:23">
       <c r="A128">
         <v>10235849</v>
       </c>
@@ -9939,7 +9952,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:23">
       <c r="A129">
         <v>10235853</v>
       </c>
@@ -10010,7 +10023,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:23">
       <c r="A130">
         <v>10235853</v>
       </c>
@@ -10081,7 +10094,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:23">
       <c r="A131">
         <v>10235853</v>
       </c>
@@ -10152,7 +10165,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:23">
       <c r="A132">
         <v>10235853</v>
       </c>
@@ -10223,7 +10236,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:23">
       <c r="A133">
         <v>10235853</v>
       </c>
@@ -10294,7 +10307,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:23">
       <c r="A134">
         <v>10235853</v>
       </c>
@@ -10365,7 +10378,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:23">
       <c r="A135">
         <v>10235853</v>
       </c>
@@ -10436,7 +10449,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:23">
       <c r="A136">
         <v>10236255</v>
       </c>
@@ -10507,7 +10520,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:23">
       <c r="A137">
         <v>10236255</v>
       </c>
@@ -10578,7 +10591,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:23">
       <c r="A138">
         <v>10236255</v>
       </c>
@@ -10649,7 +10662,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:23">
       <c r="A139">
         <v>10236255</v>
       </c>
@@ -10720,7 +10733,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:23">
       <c r="A140">
         <v>10243734</v>
       </c>
@@ -10791,7 +10804,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:23">
       <c r="A141">
         <v>10243734</v>
       </c>
@@ -10862,7 +10875,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:23">
       <c r="A142">
         <v>10243734</v>
       </c>
@@ -10933,7 +10946,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:23">
       <c r="A143">
         <v>10243734</v>
       </c>
@@ -11004,7 +11017,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:23">
       <c r="A144">
         <v>10243734</v>
       </c>
@@ -11075,7 +11088,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:23">
       <c r="A145">
         <v>10243734</v>
       </c>
@@ -11146,7 +11159,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:23">
       <c r="A146">
         <v>10244528</v>
       </c>
@@ -11217,7 +11230,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:23">
       <c r="A147">
         <v>10244528</v>
       </c>
@@ -11288,7 +11301,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:23">
       <c r="A148">
         <v>10244528</v>
       </c>
@@ -11359,7 +11372,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:23">
       <c r="A149">
         <v>10244528</v>
       </c>
@@ -11430,7 +11443,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:23">
       <c r="A150">
         <v>10244528</v>
       </c>
@@ -11501,7 +11514,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:23">
       <c r="A151">
         <v>10245034</v>
       </c>
@@ -11572,7 +11585,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:23">
       <c r="A152">
         <v>10245034</v>
       </c>
@@ -11643,7 +11656,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:23">
       <c r="A153">
         <v>10245034</v>
       </c>
@@ -11714,7 +11727,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:23">
       <c r="A154">
         <v>10245034</v>
       </c>
@@ -11785,7 +11798,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" spans="1:23">
       <c r="A155">
         <v>10245034</v>
       </c>
@@ -11856,7 +11869,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" spans="1:23">
       <c r="A156">
         <v>10245034</v>
       </c>
@@ -11927,7 +11940,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" spans="1:23">
       <c r="A157">
         <v>10245178</v>
       </c>
@@ -11998,7 +12011,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" spans="1:23">
       <c r="A158">
         <v>10245178</v>
       </c>
@@ -12069,7 +12082,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:23">
       <c r="A159">
         <v>10245178</v>
       </c>
@@ -12140,7 +12153,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:23">
       <c r="A160">
         <v>10245178</v>
       </c>
@@ -12211,7 +12224,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="1:23">
       <c r="A161">
         <v>10245178</v>
       </c>
@@ -12282,7 +12295,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="1:23">
       <c r="A162">
         <v>10245186</v>
       </c>
@@ -12353,7 +12366,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="1:23">
       <c r="A163">
         <v>10245186</v>
       </c>
@@ -12424,7 +12437,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="1:23">
       <c r="A164">
         <v>10245186</v>
       </c>
@@ -12495,7 +12508,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="1:23">
       <c r="A165">
         <v>10245186</v>
       </c>
@@ -12566,7 +12579,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="1:23">
       <c r="A166">
         <v>10245186</v>
       </c>
@@ -12637,7 +12650,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" spans="1:23">
       <c r="A167">
         <v>10245273</v>
       </c>
@@ -12708,7 +12721,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" spans="1:23">
       <c r="A168">
         <v>10245273</v>
       </c>
@@ -12779,7 +12792,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" spans="1:23">
       <c r="A169">
         <v>10245273</v>
       </c>
@@ -12850,7 +12863,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" spans="1:23">
       <c r="A170">
         <v>10245273</v>
       </c>
@@ -12921,7 +12934,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" spans="1:23">
       <c r="A171">
         <v>10245273</v>
       </c>
@@ -12992,7 +13005,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" spans="1:23">
       <c r="A172">
         <v>10245277</v>
       </c>
@@ -13063,7 +13076,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" spans="1:23">
       <c r="A173">
         <v>10245277</v>
       </c>
@@ -13134,7 +13147,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" spans="1:23">
       <c r="A174">
         <v>10245277</v>
       </c>
@@ -13205,7 +13218,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" spans="1:23">
       <c r="A175">
         <v>10245277</v>
       </c>
@@ -13276,7 +13289,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" spans="1:23">
       <c r="A176">
         <v>10245477</v>
       </c>
@@ -13347,7 +13360,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" spans="1:23">
       <c r="A177">
         <v>10245477</v>
       </c>
@@ -13418,7 +13431,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" spans="1:23">
       <c r="A178">
         <v>10245477</v>
       </c>
@@ -13489,7 +13502,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" spans="1:23">
       <c r="A179">
         <v>10245477</v>
       </c>
@@ -13560,7 +13573,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" spans="1:23">
       <c r="A180">
         <v>10245477</v>
       </c>
@@ -13631,7 +13644,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" spans="1:23">
       <c r="A181">
         <v>10245536</v>
       </c>
@@ -13702,7 +13715,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" spans="1:23">
       <c r="A182">
         <v>10245569</v>
       </c>
@@ -13773,7 +13786,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="183">
+    <row r="183" spans="1:23">
       <c r="A183">
         <v>10245569</v>
       </c>
@@ -13844,7 +13857,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" spans="1:23">
       <c r="A184">
         <v>10245569</v>
       </c>
@@ -13915,7 +13928,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" spans="1:23">
       <c r="A185">
         <v>10245569</v>
       </c>
@@ -13986,7 +13999,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" spans="1:23">
       <c r="A186">
         <v>10245569</v>
       </c>
@@ -14057,7 +14070,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="187">
+    <row r="187" spans="1:23">
       <c r="A187">
         <v>10245577</v>
       </c>
@@ -14128,7 +14141,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="188">
+    <row r="188" spans="1:23">
       <c r="A188">
         <v>10245577</v>
       </c>
@@ -14199,7 +14212,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" spans="1:23">
       <c r="A189">
         <v>10245577</v>
       </c>
@@ -14270,7 +14283,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" spans="1:23">
       <c r="A190">
         <v>10245577</v>
       </c>
@@ -14341,7 +14354,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" spans="1:23">
       <c r="A191">
         <v>10245584</v>
       </c>
@@ -14412,7 +14425,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" spans="1:23">
       <c r="A192">
         <v>10245584</v>
       </c>
@@ -14483,7 +14496,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" spans="1:23">
       <c r="A193">
         <v>10245584</v>
       </c>
@@ -14554,7 +14567,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" spans="1:23">
       <c r="A194">
         <v>10245584</v>
       </c>
@@ -14625,7 +14638,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" spans="1:23">
       <c r="A195">
         <v>10245817</v>
       </c>
@@ -14696,7 +14709,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" spans="1:23">
       <c r="A196">
         <v>10245817</v>
       </c>
@@ -14767,7 +14780,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" spans="1:23">
       <c r="A197">
         <v>10245817</v>
       </c>
@@ -14838,7 +14851,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="198">
+    <row r="198" spans="1:23">
       <c r="A198">
         <v>10245817</v>
       </c>
@@ -14909,7 +14922,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="199">
+    <row r="199" spans="1:23">
       <c r="A199">
         <v>10245977</v>
       </c>
@@ -14980,7 +14993,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" spans="1:23">
       <c r="A200">
         <v>10245977</v>
       </c>
@@ -15051,7 +15064,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" spans="1:23">
       <c r="A201">
         <v>10245977</v>
       </c>
@@ -15122,7 +15135,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="202">
+    <row r="202" spans="1:23">
       <c r="A202">
         <v>10245977</v>
       </c>
@@ -15193,7 +15206,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="203">
+    <row r="203" spans="1:23">
       <c r="A203">
         <v>10245991</v>
       </c>
@@ -15264,7 +15277,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="204">
+    <row r="204" spans="1:23">
       <c r="A204">
         <v>10245991</v>
       </c>
@@ -15335,7 +15348,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="205">
+    <row r="205" spans="1:23">
       <c r="A205">
         <v>10245991</v>
       </c>
@@ -15406,7 +15419,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="206">
+    <row r="206" spans="1:23">
       <c r="A206">
         <v>10245991</v>
       </c>
@@ -15477,7 +15490,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="207">
+    <row r="207" spans="1:23">
       <c r="A207">
         <v>10246003</v>
       </c>
@@ -15548,7 +15561,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="208">
+    <row r="208" spans="1:23">
       <c r="A208">
         <v>10246003</v>
       </c>
@@ -15619,7 +15632,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="209">
+    <row r="209" spans="1:23">
       <c r="A209">
         <v>10246003</v>
       </c>
@@ -15690,7 +15703,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="210">
+    <row r="210" spans="1:23">
       <c r="A210">
         <v>10246003</v>
       </c>
@@ -15761,7 +15774,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="211">
+    <row r="211" spans="1:23">
       <c r="A211">
         <v>10246003</v>
       </c>
@@ -15832,7 +15845,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="212">
+    <row r="212" spans="1:23">
       <c r="A212">
         <v>10246003</v>
       </c>
@@ -15903,7 +15916,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="213">
+    <row r="213" spans="1:23">
       <c r="A213">
         <v>10246012</v>
       </c>
@@ -15974,7 +15987,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="214">
+    <row r="214" spans="1:23">
       <c r="A214">
         <v>10246012</v>
       </c>
@@ -16045,7 +16058,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="215">
+    <row r="215" spans="1:23">
       <c r="A215">
         <v>10246050</v>
       </c>
@@ -16116,7 +16129,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="216">
+    <row r="216" spans="1:23">
       <c r="A216">
         <v>10246050</v>
       </c>
@@ -16187,7 +16200,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="217">
+    <row r="217" spans="1:23">
       <c r="A217">
         <v>10246050</v>
       </c>
@@ -16258,7 +16271,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="218">
+    <row r="218" spans="1:23">
       <c r="A218">
         <v>10246050</v>
       </c>
@@ -16329,7 +16342,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="219">
+    <row r="219" spans="1:23">
       <c r="A219">
         <v>10246161</v>
       </c>
@@ -16400,7 +16413,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="220">
+    <row r="220" spans="1:23">
       <c r="A220">
         <v>10246161</v>
       </c>
@@ -16471,7 +16484,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="221">
+    <row r="221" spans="1:23">
       <c r="A221">
         <v>10246161</v>
       </c>
@@ -16542,7 +16555,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="222">
+    <row r="222" spans="1:23">
       <c r="A222">
         <v>10246161</v>
       </c>
@@ -16613,7 +16626,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="223">
+    <row r="223" spans="1:23">
       <c r="A223">
         <v>10246161</v>
       </c>
@@ -16684,7 +16697,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="224">
+    <row r="224" spans="1:23">
       <c r="A224">
         <v>10246220</v>
       </c>
@@ -16755,7 +16768,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="225">
+    <row r="225" spans="1:23">
       <c r="A225">
         <v>10246220</v>
       </c>
@@ -16826,7 +16839,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="226">
+    <row r="226" spans="1:23">
       <c r="A226">
         <v>10246220</v>
       </c>
@@ -16897,7 +16910,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="227">
+    <row r="227" spans="1:23">
       <c r="A227">
         <v>10246220</v>
       </c>
@@ -16968,7 +16981,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="228">
+    <row r="228" spans="1:23">
       <c r="A228">
         <v>10246220</v>
       </c>
@@ -17039,7 +17052,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="229">
+    <row r="229" spans="1:23">
       <c r="A229">
         <v>10246457</v>
       </c>
@@ -17110,7 +17123,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="230">
+    <row r="230" spans="1:23">
       <c r="A230">
         <v>10246457</v>
       </c>
@@ -17181,7 +17194,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="231">
+    <row r="231" spans="1:23">
       <c r="A231">
         <v>10246457</v>
       </c>
@@ -17252,7 +17265,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" spans="1:23">
       <c r="A232">
         <v>10247010</v>
       </c>
@@ -17323,7 +17336,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="233">
+    <row r="233" spans="1:23">
       <c r="A233">
         <v>10247010</v>
       </c>
@@ -17394,7 +17407,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="234">
+    <row r="234" spans="1:23">
       <c r="A234">
         <v>10247010</v>
       </c>
@@ -17465,7 +17478,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="235">
+    <row r="235" spans="1:23">
       <c r="A235">
         <v>10247010</v>
       </c>
@@ -17536,7 +17549,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="236">
+    <row r="236" spans="1:23">
       <c r="A236">
         <v>10247081</v>
       </c>
@@ -17607,7 +17620,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="237">
+    <row r="237" spans="1:23">
       <c r="A237">
         <v>10247251</v>
       </c>
@@ -17678,7 +17691,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="238">
+    <row r="238" spans="1:23">
       <c r="A238">
         <v>10247251</v>
       </c>
@@ -17749,7 +17762,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="239">
+    <row r="239" spans="1:23">
       <c r="A239">
         <v>10247251</v>
       </c>
@@ -17820,7 +17833,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="240">
+    <row r="240" spans="1:23">
       <c r="A240">
         <v>10247251</v>
       </c>
@@ -17891,7 +17904,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="241">
+    <row r="241" spans="1:23">
       <c r="A241">
         <v>10247251</v>
       </c>
@@ -17962,7 +17975,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="242">
+    <row r="242" spans="1:23">
       <c r="A242">
         <v>10247251</v>
       </c>
@@ -18033,7 +18046,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="243">
+    <row r="243" spans="1:23">
       <c r="A243">
         <v>10247375</v>
       </c>
@@ -18104,7 +18117,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="244">
+    <row r="244" spans="1:23">
       <c r="A244">
         <v>10247375</v>
       </c>
@@ -18175,7 +18188,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="245">
+    <row r="245" spans="1:23">
       <c r="A245">
         <v>10247375</v>
       </c>
@@ -18246,7 +18259,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="246">
+    <row r="246" spans="1:23">
       <c r="A246">
         <v>10247447</v>
       </c>
@@ -18317,7 +18330,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="247">
+    <row r="247" spans="1:23">
       <c r="A247">
         <v>10247447</v>
       </c>
@@ -18388,7 +18401,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="248">
+    <row r="248" spans="1:23">
       <c r="A248">
         <v>10247447</v>
       </c>
@@ -18459,7 +18472,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="249">
+    <row r="249" spans="1:23">
       <c r="A249">
         <v>10247447</v>
       </c>
@@ -18530,7 +18543,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="250">
+    <row r="250" spans="1:23">
       <c r="A250">
         <v>10248065</v>
       </c>
@@ -18601,7 +18614,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="251">
+    <row r="251" spans="1:23">
       <c r="A251">
         <v>10248065</v>
       </c>
@@ -18672,7 +18685,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="252">
+    <row r="252" spans="1:23">
       <c r="A252">
         <v>10248065</v>
       </c>
@@ -18743,7 +18756,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" spans="1:23">
       <c r="A253">
         <v>10248065</v>
       </c>
@@ -18814,7 +18827,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="254">
+    <row r="254" spans="1:23">
       <c r="A254">
         <v>10248065</v>
       </c>
@@ -18885,7 +18898,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="255">
+    <row r="255" spans="1:23">
       <c r="A255">
         <v>10248065</v>
       </c>
@@ -18956,7 +18969,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="256">
+    <row r="256" spans="1:23">
       <c r="A256">
         <v>10248166</v>
       </c>
@@ -19027,7 +19040,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="257">
+    <row r="257" spans="1:23">
       <c r="A257">
         <v>10248170</v>
       </c>
@@ -19098,7 +19111,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="258">
+    <row r="258" spans="1:23">
       <c r="A258">
         <v>10248732</v>
       </c>
@@ -19169,7 +19182,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="259">
+    <row r="259" spans="1:23">
       <c r="A259">
         <v>10251998</v>
       </c>
@@ -19240,7 +19253,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" spans="1:23">
       <c r="A260">
         <v>10251998</v>
       </c>
@@ -19311,7 +19324,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="261">
+    <row r="261" spans="1:23">
       <c r="A261">
         <v>10253018</v>
       </c>
@@ -19382,7 +19395,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="262">
+    <row r="262" spans="1:23">
       <c r="A262">
         <v>10253018</v>
       </c>
@@ -19453,7 +19466,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" spans="1:23">
       <c r="A263">
         <v>10253047</v>
       </c>
@@ -19524,7 +19537,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="264">
+    <row r="264" spans="1:23">
       <c r="A264">
         <v>10253062</v>
       </c>
@@ -19595,7 +19608,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="265">
+    <row r="265" spans="1:23">
       <c r="A265">
         <v>10253062</v>
       </c>
@@ -19666,7 +19679,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="266">
+    <row r="266" spans="1:23">
       <c r="A266">
         <v>10253080</v>
       </c>
@@ -19737,7 +19750,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="267">
+    <row r="267" spans="1:23">
       <c r="A267">
         <v>10254574</v>
       </c>
@@ -19808,7 +19821,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="268">
+    <row r="268" spans="1:23">
       <c r="A268">
         <v>10254807</v>
       </c>
@@ -19879,7 +19892,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="269">
+    <row r="269" spans="1:23">
       <c r="A269">
         <v>10254809</v>
       </c>
@@ -19950,7 +19963,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="270">
+    <row r="270" spans="1:23">
       <c r="A270">
         <v>10266349</v>
       </c>
@@ -20021,7 +20034,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="271">
+    <row r="271" spans="1:23">
       <c r="A271">
         <v>10304035</v>
       </c>
@@ -20094,13 +20107,14 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="T2:V2"/>
+    <mergeCell ref="W2:W3"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="O2:S2"/>
-    <mergeCell ref="T2:V2"/>
-    <mergeCell ref="W2:W3"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>